<commit_message>
update and reorganisation of reflectance information into another repo
</commit_message>
<xml_diff>
--- a/data/biomass/AV/Aveiro_grid_info_final.xlsx
+++ b/data/biomass/AV/Aveiro_grid_info_final.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Laurent\CONTRATS\2024 REWRITE\Aveiro 2025\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\REWRITE\Field_data\seagrass_carbon_2025\data\biomass\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F023D20A-4EC7-4C2D-9EC8-F9B93BE1ACE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -21,9 +20,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">data!$A$1:$O$100</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'seagrass biomass'!$A$1:$F$165</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId4"/>
+    <pivotCache cacheId="8" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -43,7 +42,7 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>tc={50A84D78-0949-442C-8B45-B42A1C631C90}</author>
     <author>tc={B1E548A4-451D-442C-8170-46B83715A7EA}</author>
@@ -52,7 +51,7 @@
     <author>tc={E989AD93-086E-4B84-BCB0-75F70F31E996}</author>
   </authors>
   <commentList>
-    <comment ref="E6" authorId="0" shapeId="0" xr:uid="{50A84D78-0949-442C-8B45-B42A1C631C90}">
+    <comment ref="E6" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -69,7 +68,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E7" authorId="1" shapeId="0" xr:uid="{B1E548A4-451D-442C-8170-46B83715A7EA}">
+    <comment ref="E7" authorId="1" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -86,7 +85,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G11" authorId="2" shapeId="0" xr:uid="{750D5695-E24D-437A-86B5-81CD1CFB106D}">
+    <comment ref="G11" authorId="2" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -103,7 +102,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G19" authorId="3" shapeId="0" xr:uid="{E50ACC29-A39A-45E8-99D8-DB2F209B5289}">
+    <comment ref="G19" authorId="3" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -120,7 +119,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G40" authorId="4" shapeId="0" xr:uid="{E989AD93-086E-4B84-BCB0-75F70F31E996}">
+    <comment ref="G40" authorId="4" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1512,11 +1511,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00&quot; &quot;[$€-40C];[Red]&quot;-&quot;#,##0.00&quot; &quot;[$€-40C]"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1664,7 +1663,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1745,16 +1744,144 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
-    <cellStyle name="Heading" xfId="2" xr:uid="{C3BF4837-8238-451A-9F43-C45BE234F655}"/>
-    <cellStyle name="Heading1" xfId="3" xr:uid="{27EA53AD-3A81-4188-B251-8EC083B37A6B}"/>
+    <cellStyle name="Heading" xfId="2"/>
+    <cellStyle name="Heading1" xfId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Result" xfId="4" xr:uid="{BF450080-4396-4D21-9F77-0A4CD9C55119}"/>
-    <cellStyle name="Result2" xfId="5" xr:uid="{AA1EA9A6-7DDA-47EB-8102-3C9BA9DF5CE3}"/>
-    <cellStyle name="Standaard 2" xfId="1" xr:uid="{60181DCC-36DD-4550-8735-D0AD608CB25F}"/>
+    <cellStyle name="Result" xfId="4"/>
+    <cellStyle name="Result2" xfId="5"/>
+    <cellStyle name="Standaard 2" xfId="1"/>
   </cellStyles>
-  <dxfs count="15">
+  <dxfs count="45">
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="6" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="6" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1836,7 +1963,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Jim de Fouw" refreshedDate="45972.547460185182" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="179" xr:uid="{F1E11D45-1A58-4FDC-B37B-E5360D53161C}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" refreshedBy="barille-l" refreshedDate="46044.482672569444" createdVersion="8" refreshedVersion="6" minRefreshableVersion="3" recordCount="179">
   <cacheSource type="worksheet">
     <worksheetSource ref="B1:E1048576" sheet="seagrass biomass"/>
   </cacheSource>
@@ -1946,7 +2073,7 @@
       </sharedItems>
     </cacheField>
     <cacheField name="dry weight (mg)" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="0" maxValue="3982"/>
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" minValue="0" maxValue="3975.8"/>
     </cacheField>
   </cacheFields>
   <extLst>
@@ -1958,7 +2085,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="179">
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" count="179">
   <r>
     <s v="10A"/>
     <x v="0"/>
@@ -1987,7 +2114,7 @@
     <s v="115AN"/>
     <x v="2"/>
     <x v="0"/>
-    <n v="3982"/>
+    <n v="3975.8"/>
   </r>
   <r>
     <s v="115BN"/>
@@ -2197,7 +2324,7 @@
     <s v="133BN"/>
     <x v="19"/>
     <x v="1"/>
-    <n v="578"/>
+    <n v="573.5"/>
   </r>
   <r>
     <s v="134AN"/>
@@ -2359,7 +2486,7 @@
     <s v="16A"/>
     <x v="33"/>
     <x v="0"/>
-    <n v="977"/>
+    <n v="871"/>
   </r>
   <r>
     <s v="16B"/>
@@ -2455,13 +2582,13 @@
     <s v="25A"/>
     <x v="41"/>
     <x v="0"/>
-    <n v="2237"/>
+    <n v="2171"/>
   </r>
   <r>
     <s v="25B"/>
     <x v="41"/>
     <x v="1"/>
-    <n v="951"/>
+    <n v="933"/>
   </r>
   <r>
     <s v="26A"/>
@@ -2551,13 +2678,13 @@
     <s v="35A"/>
     <x v="49"/>
     <x v="0"/>
-    <n v="209"/>
+    <n v="206.02"/>
   </r>
   <r>
     <s v="35B"/>
     <x v="49"/>
     <x v="1"/>
-    <n v="248"/>
+    <n v="212.4"/>
   </r>
   <r>
     <s v="36A"/>
@@ -3037,7 +3164,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B7D7D528-D861-4B64-AC95-A0A3C3AC63F4}" name="Draaitabel1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Waarden" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="Draaitabel1" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Waarden" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="G1:K93" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField showAll="0"/>
@@ -3445,25 +3572,25 @@
     <dataField name="Average of dry weight (mg)" fld="3" subtotal="average" baseField="1" baseItem="0"/>
   </dataFields>
   <formats count="15">
-    <format dxfId="14">
+    <format dxfId="44">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="13">
+    <format dxfId="43">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="12">
+    <format dxfId="42">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="11">
+    <format dxfId="41">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="10">
+    <format dxfId="40">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="9">
+    <format dxfId="39">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="8">
+    <format dxfId="38">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="50">
@@ -3521,7 +3648,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="7">
+    <format dxfId="37">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="29">
@@ -3558,20 +3685,20 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="6">
+    <format dxfId="36">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="5">
+    <format dxfId="35">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="4">
+    <format dxfId="34">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="3">
+    <format dxfId="33">
       <pivotArea dataOnly="0" fieldPosition="0">
         <references count="1">
           <reference field="1" count="1">
@@ -3580,7 +3707,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="2">
+    <format dxfId="32">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="1">
@@ -3589,7 +3716,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="1">
+    <format dxfId="31">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="1">
@@ -3598,7 +3725,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="0">
+    <format dxfId="30">
       <pivotArea dataOnly="0" fieldPosition="0">
         <references count="1">
           <reference field="1" count="1">
@@ -3621,7 +3748,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -3696,23 +3823,6 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -3748,23 +3858,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -3960,9 +4053,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:O100"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="5" width="8.7109375" style="2"/>
     <col min="6" max="7" width="15.5703125" style="2" customWidth="1"/>
@@ -3976,7 +4069,7 @@
     <col min="17" max="16384" width="8.7109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="1" customFormat="1">
+    <row r="1" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4023,7 +4116,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="2" spans="1:15">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>111</v>
       </c>
@@ -4063,7 +4156,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>112</v>
       </c>
@@ -4103,7 +4196,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>111</v>
       </c>
@@ -4149,7 +4242,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>111</v>
       </c>
@@ -4189,7 +4282,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>111</v>
       </c>
@@ -4229,7 +4322,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="7" spans="1:15">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>111</v>
       </c>
@@ -4269,7 +4362,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>111</v>
       </c>
@@ -4309,7 +4402,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="9" spans="1:15">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>112</v>
       </c>
@@ -4349,7 +4442,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>112</v>
       </c>
@@ -4389,7 +4482,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="11" spans="1:15">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>111</v>
       </c>
@@ -4429,7 +4522,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="12" spans="1:15">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>112</v>
       </c>
@@ -4469,7 +4562,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="13" spans="1:15">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>112</v>
       </c>
@@ -4509,7 +4602,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="14" spans="1:15">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>111</v>
       </c>
@@ -4549,7 +4642,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="15" spans="1:15">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>111</v>
       </c>
@@ -4589,7 +4682,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="16" spans="1:15">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>112</v>
       </c>
@@ -4629,7 +4722,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="17" spans="1:15">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>111</v>
       </c>
@@ -4659,7 +4752,7 @@
       </c>
       <c r="J17" s="5">
         <f>VLOOKUP($F17,'seagrass biomass'!$G:$L,2,FALSE)</f>
-        <v>977</v>
+        <v>871</v>
       </c>
       <c r="K17" s="5">
         <f>VLOOKUP($F17,'seagrass biomass'!$G:$L,3,FALSE)</f>
@@ -4672,7 +4765,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="18" spans="1:15">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>111</v>
       </c>
@@ -4712,7 +4805,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="19" spans="1:15">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>112</v>
       </c>
@@ -4752,7 +4845,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="20" spans="1:15">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>111</v>
       </c>
@@ -4801,7 +4894,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="21" spans="1:15">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>111</v>
       </c>
@@ -4841,7 +4934,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="22" spans="1:15">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>112</v>
       </c>
@@ -4881,7 +4974,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="23" spans="1:15">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>112</v>
       </c>
@@ -4921,7 +5014,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="24" spans="1:15">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>111</v>
       </c>
@@ -4967,7 +5060,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="25" spans="1:15">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>112</v>
       </c>
@@ -5013,7 +5106,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="26" spans="1:15">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>111</v>
       </c>
@@ -5043,11 +5136,11 @@
       </c>
       <c r="J26" s="16">
         <f>VLOOKUP($F26,'seagrass biomass'!$G:$L,2,FALSE)</f>
-        <v>2237</v>
+        <v>2171</v>
       </c>
       <c r="K26" s="16">
         <f>VLOOKUP($F26,'seagrass biomass'!$G:$L,3,FALSE)</f>
-        <v>951</v>
+        <v>933</v>
       </c>
       <c r="L26" s="16" t="s">
         <v>386</v>
@@ -5059,7 +5152,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="27" spans="1:15">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>111</v>
       </c>
@@ -5105,7 +5198,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="28" spans="1:15">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>112</v>
       </c>
@@ -5145,7 +5238,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="29" spans="1:15">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>111</v>
       </c>
@@ -5185,7 +5278,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="30" spans="1:15">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>112</v>
       </c>
@@ -5231,7 +5324,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="31" spans="1:15">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>111</v>
       </c>
@@ -5277,7 +5370,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="32" spans="1:15">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>112</v>
       </c>
@@ -5317,7 +5410,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="33" spans="1:14">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>112</v>
       </c>
@@ -5357,7 +5450,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="34" spans="1:14">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>111</v>
       </c>
@@ -5397,7 +5490,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="35" spans="1:14">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>111</v>
       </c>
@@ -5443,7 +5536,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="36" spans="1:14">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>112</v>
       </c>
@@ -5473,11 +5566,11 @@
       </c>
       <c r="J36" s="16">
         <f>VLOOKUP($F36,'seagrass biomass'!$G:$L,2,FALSE)</f>
-        <v>209</v>
+        <v>206.02</v>
       </c>
       <c r="K36" s="16">
         <f>VLOOKUP($F36,'seagrass biomass'!$G:$L,3,FALSE)</f>
-        <v>248</v>
+        <v>212.4</v>
       </c>
       <c r="L36" s="16" t="s">
         <v>386</v>
@@ -5489,7 +5582,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="37" spans="1:14">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>111</v>
       </c>
@@ -5535,7 +5628,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="38" spans="1:14">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>111</v>
       </c>
@@ -5575,7 +5668,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="39" spans="1:14">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>112</v>
       </c>
@@ -5615,7 +5708,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="40" spans="1:14">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>111</v>
       </c>
@@ -5661,7 +5754,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="41" spans="1:14">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>111</v>
       </c>
@@ -5707,7 +5800,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="42" spans="1:14">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>112</v>
       </c>
@@ -5747,7 +5840,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="43" spans="1:14">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>111</v>
       </c>
@@ -5787,7 +5880,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="44" spans="1:14">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>111</v>
       </c>
@@ -5828,7 +5921,7 @@
         <v>NIOZ lab</v>
       </c>
     </row>
-    <row r="45" spans="1:14">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>112</v>
       </c>
@@ -5868,7 +5961,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="46" spans="1:14">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>111</v>
       </c>
@@ -5908,7 +6001,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="47" spans="1:14">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>111</v>
       </c>
@@ -5948,7 +6041,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="48" spans="1:14">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>112</v>
       </c>
@@ -5988,7 +6081,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="49" spans="1:15">
+    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>112</v>
       </c>
@@ -6028,7 +6121,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="50" spans="1:15">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>111</v>
       </c>
@@ -6071,7 +6164,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="51" spans="1:15">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>111</v>
       </c>
@@ -6112,7 +6205,7 @@
         <v>NIOZ lab</v>
       </c>
     </row>
-    <row r="52" spans="1:15">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>112</v>
       </c>
@@ -6152,7 +6245,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="53" spans="1:15">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>111</v>
       </c>
@@ -6192,7 +6285,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="54" spans="1:15">
+    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>112</v>
       </c>
@@ -6232,7 +6325,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="55" spans="1:15">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>111</v>
       </c>
@@ -6273,7 +6366,7 @@
         <v>NIOZ lab</v>
       </c>
     </row>
-    <row r="56" spans="1:15">
+    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>112</v>
       </c>
@@ -6314,7 +6407,7 @@
         <v>NIOZ lab</v>
       </c>
     </row>
-    <row r="57" spans="1:15">
+    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>111</v>
       </c>
@@ -6354,7 +6447,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="58" spans="1:15">
+    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>111</v>
       </c>
@@ -6403,7 +6496,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="59" spans="1:15">
+    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>111</v>
       </c>
@@ -6433,7 +6526,7 @@
       </c>
       <c r="J59" s="5">
         <f>VLOOKUP($F59,'seagrass biomass'!$G:$L,2,FALSE)</f>
-        <v>3982</v>
+        <v>3975.8</v>
       </c>
       <c r="K59" s="5">
         <f>VLOOKUP($F59,'seagrass biomass'!$G:$L,3,FALSE)</f>
@@ -6443,7 +6536,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="60" spans="1:15">
+    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>111</v>
       </c>
@@ -6483,7 +6576,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="61" spans="1:15">
+    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>112</v>
       </c>
@@ -6529,7 +6622,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="62" spans="1:15">
+    <row r="62" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>111</v>
       </c>
@@ -6576,7 +6669,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="63" spans="1:15">
+    <row r="63" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>111</v>
       </c>
@@ -6622,7 +6715,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="64" spans="1:15">
+    <row r="64" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>111</v>
       </c>
@@ -6665,7 +6758,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="65" spans="1:15">
+    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>111</v>
       </c>
@@ -6711,7 +6804,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="66" spans="1:15">
+    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>112</v>
       </c>
@@ -6757,7 +6850,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="67" spans="1:15">
+    <row r="67" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>111</v>
       </c>
@@ -6806,7 +6899,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="68" spans="1:15">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>112</v>
       </c>
@@ -6846,7 +6939,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="69" spans="1:15">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
         <v>112</v>
       </c>
@@ -6886,7 +6979,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="70" spans="1:15">
+    <row r="70" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>111</v>
       </c>
@@ -6926,7 +7019,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="71" spans="1:15">
+    <row r="71" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>112</v>
       </c>
@@ -6966,7 +7059,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="72" spans="1:15">
+    <row r="72" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>111</v>
       </c>
@@ -7006,7 +7099,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="73" spans="1:15">
+    <row r="73" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>111</v>
       </c>
@@ -7056,7 +7149,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="74" spans="1:15">
+    <row r="74" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>112</v>
       </c>
@@ -7105,7 +7198,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="75" spans="1:15">
+    <row r="75" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
         <v>111</v>
       </c>
@@ -7152,7 +7245,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="76" spans="1:15">
+    <row r="76" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>111</v>
       </c>
@@ -7201,7 +7294,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="77" spans="1:15">
+    <row r="77" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>112</v>
       </c>
@@ -7235,13 +7328,13 @@
       </c>
       <c r="K77" s="5">
         <f>VLOOKUP($F77,'seagrass biomass'!$G:$L,3,FALSE)</f>
-        <v>578</v>
+        <v>573.5</v>
       </c>
       <c r="L77" s="5" t="s">
         <v>386</v>
       </c>
     </row>
-    <row r="78" spans="1:15">
+    <row r="78" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>112</v>
       </c>
@@ -7281,7 +7374,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="79" spans="1:15">
+    <row r="79" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>111</v>
       </c>
@@ -7321,7 +7414,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="80" spans="1:15">
+    <row r="80" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>112</v>
       </c>
@@ -7362,7 +7455,7 @@
         <v>NIOZ lab</v>
       </c>
     </row>
-    <row r="81" spans="1:15">
+    <row r="81" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
         <v>111</v>
       </c>
@@ -7402,7 +7495,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="82" spans="1:15">
+    <row r="82" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>112</v>
       </c>
@@ -7442,7 +7535,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="83" spans="1:15">
+    <row r="83" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
         <v>111</v>
       </c>
@@ -7483,7 +7576,7 @@
         <v>NIOZ lab</v>
       </c>
     </row>
-    <row r="84" spans="1:15">
+    <row r="84" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
         <v>111</v>
       </c>
@@ -7523,7 +7616,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="85" spans="1:15">
+    <row r="85" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
         <v>111</v>
       </c>
@@ -7563,7 +7656,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="86" spans="1:15">
+    <row r="86" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
         <v>111</v>
       </c>
@@ -7603,7 +7696,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="87" spans="1:15">
+    <row r="87" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
         <v>111</v>
       </c>
@@ -7623,7 +7716,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="88" spans="1:15">
+    <row r="88" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
         <v>111</v>
       </c>
@@ -7643,7 +7736,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="89" spans="1:15">
+    <row r="89" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
         <v>111</v>
       </c>
@@ -7663,7 +7756,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="90" spans="1:15">
+    <row r="90" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>111</v>
       </c>
@@ -7683,7 +7776,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="91" spans="1:15">
+    <row r="91" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
         <v>111</v>
       </c>
@@ -7703,7 +7796,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="92" spans="1:15">
+    <row r="92" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
         <v>111</v>
       </c>
@@ -7723,7 +7816,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="93" spans="1:15">
+    <row r="93" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
         <v>111</v>
       </c>
@@ -7743,7 +7836,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="94" spans="1:15">
+    <row r="94" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
         <v>112</v>
       </c>
@@ -7763,7 +7856,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="95" spans="1:15">
+    <row r="95" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
         <v>112</v>
       </c>
@@ -7783,7 +7876,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="96" spans="1:15">
+    <row r="96" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
         <v>112</v>
       </c>
@@ -7803,7 +7896,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="97" spans="1:9">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
         <v>112</v>
       </c>
@@ -7823,7 +7916,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="98" spans="1:9">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
         <v>111</v>
       </c>
@@ -7843,7 +7936,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="99" spans="1:9">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
         <v>112</v>
       </c>
@@ -7863,7 +7956,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="100" spans="1:9">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
         <v>112</v>
       </c>
@@ -7884,8 +7977,8 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O100" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:O100">
+  <autoFilter ref="A1:O100"/>
+  <sortState ref="A2:O100">
     <sortCondition ref="F2:F100"/>
   </sortState>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -7895,21 +7988,21 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60289AD6-9204-4C5F-9F5B-57B3483DE391}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:X179"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="8.7109375" style="2"/>
     <col min="5" max="6" width="15.140625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="23.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12" style="2" bestFit="1" customWidth="1"/>
     <col min="12" max="16384" width="8.7109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>374</v>
       </c>
@@ -7941,7 +8034,7 @@
       <c r="Q1" s="8"/>
       <c r="R1" s="8"/>
     </row>
-    <row r="2" spans="1:18">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -7982,7 +8075,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="3" spans="1:18">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -8001,14 +8094,14 @@
       <c r="G3" s="15">
         <v>2025003</v>
       </c>
-      <c r="H3" s="15">
+      <c r="H3" s="29">
         <v>315</v>
       </c>
-      <c r="I3" s="15">
+      <c r="I3" s="29">
         <v>250</v>
       </c>
-      <c r="J3" s="15"/>
-      <c r="K3" s="15">
+      <c r="J3" s="29"/>
+      <c r="K3" s="29">
         <v>282.5</v>
       </c>
       <c r="O3" s="7"/>
@@ -8018,7 +8111,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="4" spans="1:18">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -8037,13 +8130,14 @@
       <c r="G4" s="2">
         <v>2025004</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="28">
         <v>42</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="28">
         <v>141</v>
       </c>
-      <c r="K4" s="2">
+      <c r="J4" s="28"/>
+      <c r="K4" s="28">
         <v>91.5</v>
       </c>
       <c r="O4" s="9" t="s">
@@ -8055,7 +8149,7 @@
       <c r="Q4" s="8"/>
       <c r="R4" s="8"/>
     </row>
-    <row r="5" spans="1:18">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -8074,13 +8168,14 @@
       <c r="G5" s="2">
         <v>2025005</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="28">
         <v>2222</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="28">
         <v>939</v>
       </c>
-      <c r="K5" s="2">
+      <c r="J5" s="28"/>
+      <c r="K5" s="28">
         <v>1580.5</v>
       </c>
       <c r="O5" s="20" t="s">
@@ -8094,7 +8189,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="6" spans="1:18">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -8108,18 +8203,20 @@
         <v>369</v>
       </c>
       <c r="E6" s="2">
-        <v>3982</v>
+        <f>3982-6.2</f>
+        <v>3975.8</v>
       </c>
       <c r="G6" s="2">
         <v>2025006</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="28">
         <v>17</v>
       </c>
-      <c r="I6" s="2">
-        <v>0</v>
-      </c>
-      <c r="K6" s="2">
+      <c r="I6" s="28">
+        <v>0</v>
+      </c>
+      <c r="J6" s="28"/>
+      <c r="K6" s="28">
         <v>8.5</v>
       </c>
       <c r="O6" s="20" t="s">
@@ -8131,7 +8228,7 @@
       <c r="Q6" s="8"/>
       <c r="R6" s="8"/>
     </row>
-    <row r="7" spans="1:18">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -8150,13 +8247,14 @@
       <c r="G7" s="2">
         <v>2025007</v>
       </c>
-      <c r="H7" s="2">
-        <v>0</v>
-      </c>
-      <c r="I7" s="2">
-        <v>0</v>
-      </c>
-      <c r="K7" s="2">
+      <c r="H7" s="28">
+        <v>0</v>
+      </c>
+      <c r="I7" s="28">
+        <v>0</v>
+      </c>
+      <c r="J7" s="28"/>
+      <c r="K7" s="28">
         <v>0</v>
       </c>
       <c r="O7" s="10" t="s">
@@ -8168,7 +8266,7 @@
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
     </row>
-    <row r="8" spans="1:18">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -8187,13 +8285,14 @@
       <c r="G8" s="2">
         <v>2025008</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="28">
         <v>2418</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="28">
         <v>1706</v>
       </c>
-      <c r="K8" s="2">
+      <c r="J8" s="28"/>
+      <c r="K8" s="28">
         <v>2062</v>
       </c>
       <c r="O8" s="10" t="s">
@@ -8205,7 +8304,7 @@
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
     </row>
-    <row r="9" spans="1:18">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -8224,25 +8323,27 @@
       <c r="G9" s="2">
         <v>2025009</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="28">
         <v>1377</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="28">
         <v>1864</v>
       </c>
-      <c r="K9" s="2">
+      <c r="J9" s="28"/>
+      <c r="K9" s="28">
         <v>1620.5</v>
       </c>
       <c r="O9" s="10" t="s">
         <v>227</v>
       </c>
       <c r="P9" s="10">
-        <v>3982</v>
+        <f>3982-6.2</f>
+        <v>3975.8</v>
       </c>
       <c r="Q9" s="8"/>
       <c r="R9" s="8"/>
     </row>
-    <row r="10" spans="1:18">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -8261,13 +8362,14 @@
       <c r="G10" s="2">
         <v>2025010</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="28">
         <v>2797</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="28">
         <v>1048</v>
       </c>
-      <c r="K10" s="2">
+      <c r="J10" s="28"/>
+      <c r="K10" s="28">
         <v>1922.5</v>
       </c>
       <c r="O10" s="10" t="s">
@@ -8279,7 +8381,7 @@
       <c r="Q10" s="8"/>
       <c r="R10" s="8"/>
     </row>
-    <row r="11" spans="1:18">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -8298,13 +8400,14 @@
       <c r="G11" s="2">
         <v>2025011</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="28">
         <v>3628</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="28">
         <v>977</v>
       </c>
-      <c r="K11" s="2">
+      <c r="J11" s="28"/>
+      <c r="K11" s="28">
         <v>2302.5</v>
       </c>
       <c r="O11" s="10" t="s">
@@ -8316,7 +8419,7 @@
       <c r="Q11" s="8"/>
       <c r="R11" s="8"/>
     </row>
-    <row r="12" spans="1:18">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -8335,13 +8438,14 @@
       <c r="G12" s="2">
         <v>2025012</v>
       </c>
-      <c r="H12" s="2">
-        <v>0</v>
-      </c>
-      <c r="I12" s="2">
-        <v>0</v>
-      </c>
-      <c r="K12" s="2">
+      <c r="H12" s="28">
+        <v>0</v>
+      </c>
+      <c r="I12" s="28">
+        <v>0</v>
+      </c>
+      <c r="J12" s="28"/>
+      <c r="K12" s="28">
         <v>0</v>
       </c>
       <c r="O12" s="10" t="s">
@@ -8353,7 +8457,7 @@
       <c r="Q12" s="8"/>
       <c r="R12" s="8"/>
     </row>
-    <row r="13" spans="1:18">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -8372,13 +8476,14 @@
       <c r="G13" s="2">
         <v>2025013</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="28">
         <v>1701</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="28">
         <v>1821</v>
       </c>
-      <c r="K13" s="2">
+      <c r="J13" s="28"/>
+      <c r="K13" s="28">
         <v>1761</v>
       </c>
       <c r="O13" s="10" t="s">
@@ -8390,7 +8495,7 @@
       <c r="Q13" s="8"/>
       <c r="R13" s="8"/>
     </row>
-    <row r="14" spans="1:18">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -8409,13 +8514,14 @@
       <c r="G14" s="2">
         <v>2025014</v>
       </c>
-      <c r="H14" s="2">
-        <v>0</v>
-      </c>
-      <c r="I14" s="2">
-        <v>0</v>
-      </c>
-      <c r="K14" s="2">
+      <c r="H14" s="28">
+        <v>0</v>
+      </c>
+      <c r="I14" s="28">
+        <v>0</v>
+      </c>
+      <c r="J14" s="28"/>
+      <c r="K14" s="28">
         <v>0</v>
       </c>
       <c r="O14" s="10" t="s">
@@ -8427,7 +8533,7 @@
       <c r="Q14" s="8"/>
       <c r="R14" s="8"/>
     </row>
-    <row r="15" spans="1:18">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -8446,13 +8552,14 @@
       <c r="G15" s="2">
         <v>2025015</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="28">
         <v>31</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="28">
         <v>189</v>
       </c>
-      <c r="K15" s="2">
+      <c r="J15" s="28"/>
+      <c r="K15" s="28">
         <v>110</v>
       </c>
       <c r="O15" s="20" t="s">
@@ -8464,7 +8571,7 @@
       <c r="Q15" s="8"/>
       <c r="R15" s="8"/>
     </row>
-    <row r="16" spans="1:18">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -8483,14 +8590,15 @@
       <c r="G16" s="2">
         <v>2025016</v>
       </c>
-      <c r="H16" s="2">
-        <v>977</v>
-      </c>
-      <c r="I16" s="2">
+      <c r="H16" s="28">
+        <v>871</v>
+      </c>
+      <c r="I16" s="28">
         <v>401</v>
       </c>
-      <c r="K16" s="2">
-        <v>689</v>
+      <c r="J16" s="28"/>
+      <c r="K16" s="28">
+        <v>636</v>
       </c>
       <c r="O16" s="20" t="s">
         <v>234</v>
@@ -8501,7 +8609,7 @@
       <c r="Q16" s="8"/>
       <c r="R16" s="8"/>
     </row>
-    <row r="17" spans="1:16">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -8520,13 +8628,14 @@
       <c r="G17" s="2">
         <v>2025017</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="28">
         <v>994</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="28">
         <v>343</v>
       </c>
-      <c r="K17" s="2">
+      <c r="J17" s="28"/>
+      <c r="K17" s="28">
         <v>668.5</v>
       </c>
       <c r="O17" s="10" t="s">
@@ -8536,7 +8645,7 @@
         <v>3628</v>
       </c>
     </row>
-    <row r="18" spans="1:16">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -8555,13 +8664,14 @@
       <c r="G18" s="2">
         <v>2025018</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="28">
         <v>2523</v>
       </c>
-      <c r="I18" s="2">
+      <c r="I18" s="28">
         <v>1219</v>
       </c>
-      <c r="K18" s="2">
+      <c r="J18" s="28"/>
+      <c r="K18" s="28">
         <v>1871</v>
       </c>
       <c r="O18" s="10" t="s">
@@ -8571,7 +8681,7 @@
         <v>977</v>
       </c>
     </row>
-    <row r="19" spans="1:16">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -8590,13 +8700,14 @@
       <c r="G19" s="2">
         <v>2025019</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="28">
         <v>2695</v>
       </c>
-      <c r="I19" s="2">
+      <c r="I19" s="28">
         <v>1160</v>
       </c>
-      <c r="K19" s="2">
+      <c r="J19" s="28"/>
+      <c r="K19" s="28">
         <v>1927.5</v>
       </c>
       <c r="O19" s="10" t="s">
@@ -8606,7 +8717,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:16">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -8625,13 +8736,14 @@
       <c r="G20" s="2">
         <v>2025021</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="28">
         <v>933</v>
       </c>
-      <c r="I20" s="2">
+      <c r="I20" s="28">
         <v>750</v>
       </c>
-      <c r="K20" s="2">
+      <c r="J20" s="28"/>
+      <c r="K20" s="28">
         <v>841.5</v>
       </c>
       <c r="O20" s="10" t="s">
@@ -8641,7 +8753,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="21" spans="1:16">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -8660,13 +8772,14 @@
       <c r="G21" s="2">
         <v>2025022</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="28">
         <v>85</v>
       </c>
-      <c r="I21" s="2">
+      <c r="I21" s="28">
         <v>719</v>
       </c>
-      <c r="K21" s="2">
+      <c r="J21" s="28"/>
+      <c r="K21" s="28">
         <v>402</v>
       </c>
       <c r="O21" s="10" t="s">
@@ -8676,7 +8789,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="22" spans="1:16">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -8695,13 +8808,14 @@
       <c r="G22" s="2">
         <v>2025023</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="28">
         <v>2790</v>
       </c>
-      <c r="I22" s="2">
+      <c r="I22" s="28">
         <v>888</v>
       </c>
-      <c r="K22" s="2">
+      <c r="J22" s="28"/>
+      <c r="K22" s="28">
         <v>1839</v>
       </c>
       <c r="O22" s="10" t="s">
@@ -8711,7 +8825,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="23" spans="1:16">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -8730,14 +8844,14 @@
       <c r="G23" s="15">
         <v>2025024</v>
       </c>
-      <c r="H23" s="15">
+      <c r="H23" s="29">
         <v>2113</v>
       </c>
-      <c r="I23" s="15">
+      <c r="I23" s="29">
         <v>675</v>
       </c>
-      <c r="J23" s="15"/>
-      <c r="K23" s="15">
+      <c r="J23" s="29"/>
+      <c r="K23" s="29">
         <v>1394</v>
       </c>
       <c r="O23" s="10" t="s">
@@ -8747,7 +8861,7 @@
         <v>2650</v>
       </c>
     </row>
-    <row r="24" spans="1:16">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -8766,14 +8880,15 @@
       <c r="G24" s="2">
         <v>2025025</v>
       </c>
-      <c r="H24" s="2">
-        <v>2237</v>
-      </c>
-      <c r="I24" s="2">
-        <v>951</v>
-      </c>
-      <c r="K24" s="2">
-        <v>1594</v>
+      <c r="H24" s="28">
+        <v>2171</v>
+      </c>
+      <c r="I24" s="28">
+        <v>933</v>
+      </c>
+      <c r="J24" s="28"/>
+      <c r="K24" s="28">
+        <v>1552</v>
       </c>
       <c r="O24" s="10" t="s">
         <v>243</v>
@@ -8782,7 +8897,7 @@
         <v>1147</v>
       </c>
     </row>
-    <row r="25" spans="1:16">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -8801,13 +8916,14 @@
       <c r="G25" s="2">
         <v>2025026</v>
       </c>
-      <c r="H25" s="2">
-        <v>0</v>
-      </c>
-      <c r="I25" s="2">
-        <v>0</v>
-      </c>
-      <c r="K25" s="2">
+      <c r="H25" s="28">
+        <v>0</v>
+      </c>
+      <c r="I25" s="28">
+        <v>0</v>
+      </c>
+      <c r="J25" s="28"/>
+      <c r="K25" s="28">
         <v>0</v>
       </c>
       <c r="O25" s="10" t="s">
@@ -8817,7 +8933,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="26" spans="1:16">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -8836,13 +8952,14 @@
       <c r="G26" s="2">
         <v>2025027</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="28">
         <v>39</v>
       </c>
-      <c r="I26" s="2">
+      <c r="I26" s="28">
         <v>161</v>
       </c>
-      <c r="K26" s="2">
+      <c r="J26" s="28"/>
+      <c r="K26" s="28">
         <v>100</v>
       </c>
       <c r="O26" s="10" t="s">
@@ -8852,7 +8969,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="27" spans="1:16">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -8871,13 +8988,14 @@
       <c r="G27" s="2">
         <v>2025028</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="28">
         <v>2715</v>
       </c>
-      <c r="I27" s="2">
+      <c r="I27" s="28">
         <v>1696</v>
       </c>
-      <c r="K27" s="2">
+      <c r="J27" s="28"/>
+      <c r="K27" s="28">
         <v>2205.5</v>
       </c>
       <c r="O27" s="10" t="s">
@@ -8887,7 +9005,7 @@
         <v>2564</v>
       </c>
     </row>
-    <row r="28" spans="1:16">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -8906,13 +9024,14 @@
       <c r="G28" s="2">
         <v>2025029</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="28">
         <v>1294</v>
       </c>
-      <c r="I28" s="2">
+      <c r="I28" s="28">
         <v>454</v>
       </c>
-      <c r="K28" s="2">
+      <c r="J28" s="28"/>
+      <c r="K28" s="28">
         <v>874</v>
       </c>
       <c r="O28" s="10" t="s">
@@ -8922,7 +9041,7 @@
         <v>2102</v>
       </c>
     </row>
-    <row r="29" spans="1:16">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -8941,13 +9060,14 @@
       <c r="G29" s="2">
         <v>2025030</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="28">
         <v>228</v>
       </c>
-      <c r="I29" s="2">
+      <c r="I29" s="28">
         <v>191</v>
       </c>
-      <c r="K29" s="2">
+      <c r="J29" s="28"/>
+      <c r="K29" s="28">
         <v>209.5</v>
       </c>
       <c r="O29" s="10" t="s">
@@ -8957,7 +9077,7 @@
         <v>1891</v>
       </c>
     </row>
-    <row r="30" spans="1:16">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -8976,13 +9096,14 @@
       <c r="G30" s="2">
         <v>2025031</v>
       </c>
-      <c r="H30" s="2">
-        <v>0</v>
-      </c>
-      <c r="I30" s="2">
-        <v>0</v>
-      </c>
-      <c r="K30" s="2">
+      <c r="H30" s="28">
+        <v>0</v>
+      </c>
+      <c r="I30" s="28">
+        <v>0</v>
+      </c>
+      <c r="J30" s="28"/>
+      <c r="K30" s="28">
         <v>0</v>
       </c>
       <c r="O30" s="10" t="s">
@@ -8992,7 +9113,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="31" spans="1:16">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>30</v>
       </c>
@@ -9011,13 +9132,14 @@
       <c r="G31" s="2">
         <v>2025034</v>
       </c>
-      <c r="H31" s="2">
-        <v>0</v>
-      </c>
-      <c r="I31" s="2">
-        <v>0</v>
-      </c>
-      <c r="K31" s="2">
+      <c r="H31" s="28">
+        <v>0</v>
+      </c>
+      <c r="I31" s="28">
+        <v>0</v>
+      </c>
+      <c r="J31" s="28"/>
+      <c r="K31" s="28">
         <v>0</v>
       </c>
       <c r="O31" s="10" t="s">
@@ -9027,7 +9149,7 @@
         <v>2057</v>
       </c>
     </row>
-    <row r="32" spans="1:16">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -9046,14 +9168,15 @@
       <c r="G32" s="2">
         <v>2025035</v>
       </c>
-      <c r="H32" s="2">
-        <v>209</v>
-      </c>
-      <c r="I32" s="2">
-        <v>248</v>
-      </c>
-      <c r="K32" s="2">
-        <v>228.5</v>
+      <c r="H32" s="28">
+        <v>206.02</v>
+      </c>
+      <c r="I32" s="28">
+        <v>212.4</v>
+      </c>
+      <c r="J32" s="28"/>
+      <c r="K32" s="28">
+        <v>209.21</v>
       </c>
       <c r="O32" s="10" t="s">
         <v>251</v>
@@ -9062,7 +9185,7 @@
         <v>1686</v>
       </c>
     </row>
-    <row r="33" spans="1:16">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>32</v>
       </c>
@@ -9081,13 +9204,14 @@
       <c r="G33" s="2">
         <v>2025036</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="28">
         <v>645</v>
       </c>
-      <c r="I33" s="2">
+      <c r="I33" s="28">
         <v>607</v>
       </c>
-      <c r="K33" s="2">
+      <c r="J33" s="28"/>
+      <c r="K33" s="28">
         <v>626</v>
       </c>
       <c r="O33" s="10" t="s">
@@ -9097,7 +9221,7 @@
         <v>926</v>
       </c>
     </row>
-    <row r="34" spans="1:16">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>33</v>
       </c>
@@ -9116,13 +9240,14 @@
       <c r="G34" s="2">
         <v>2025037</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="28">
         <v>1871</v>
       </c>
-      <c r="I34" s="2">
+      <c r="I34" s="28">
         <v>1585</v>
       </c>
-      <c r="K34" s="2">
+      <c r="J34" s="28"/>
+      <c r="K34" s="28">
         <v>1728</v>
       </c>
       <c r="O34" s="10" t="s">
@@ -9132,7 +9257,7 @@
         <v>1187</v>
       </c>
     </row>
-    <row r="35" spans="1:16">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>34</v>
       </c>
@@ -9151,13 +9276,14 @@
       <c r="G35" s="2">
         <v>2025038</v>
       </c>
-      <c r="H35" s="2">
+      <c r="H35" s="28">
         <v>1642</v>
       </c>
-      <c r="I35" s="2">
+      <c r="I35" s="28">
         <v>1381</v>
       </c>
-      <c r="K35" s="2">
+      <c r="J35" s="28"/>
+      <c r="K35" s="28">
         <v>1511.5</v>
       </c>
       <c r="O35" s="10" t="s">
@@ -9167,7 +9293,7 @@
         <v>2434</v>
       </c>
     </row>
-    <row r="36" spans="1:16">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>35</v>
       </c>
@@ -9186,13 +9312,14 @@
       <c r="G36" s="2">
         <v>2025040</v>
       </c>
-      <c r="H36" s="2">
-        <v>0</v>
-      </c>
-      <c r="I36" s="2">
-        <v>0</v>
-      </c>
-      <c r="K36" s="2">
+      <c r="H36" s="28">
+        <v>0</v>
+      </c>
+      <c r="I36" s="28">
+        <v>0</v>
+      </c>
+      <c r="J36" s="28"/>
+      <c r="K36" s="28">
         <v>0</v>
       </c>
       <c r="O36" s="10" t="s">
@@ -9202,7 +9329,7 @@
         <v>1076</v>
       </c>
     </row>
-    <row r="37" spans="1:16">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>36</v>
       </c>
@@ -9221,13 +9348,14 @@
       <c r="G37" s="2">
         <v>2025081</v>
       </c>
-      <c r="H37" s="2">
+      <c r="H37" s="28">
         <v>2745</v>
       </c>
-      <c r="I37" s="2">
+      <c r="I37" s="28">
         <v>1244</v>
       </c>
-      <c r="K37" s="2">
+      <c r="J37" s="28"/>
+      <c r="K37" s="28">
         <v>1994.5</v>
       </c>
       <c r="O37" s="20" t="s">
@@ -9237,7 +9365,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="38" spans="1:16">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <v>37</v>
       </c>
@@ -9256,13 +9384,14 @@
       <c r="G38" s="2">
         <v>2025082</v>
       </c>
-      <c r="H38" s="2">
+      <c r="H38" s="28">
         <v>400</v>
       </c>
-      <c r="I38" s="2">
+      <c r="I38" s="28">
         <v>338</v>
       </c>
-      <c r="K38" s="2">
+      <c r="J38" s="28"/>
+      <c r="K38" s="28">
         <v>369</v>
       </c>
       <c r="O38" s="20" t="s">
@@ -9272,7 +9401,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="39" spans="1:16">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>38</v>
       </c>
@@ -9291,13 +9420,14 @@
       <c r="G39" s="2">
         <v>2025084</v>
       </c>
-      <c r="H39" s="2">
+      <c r="H39" s="28">
         <v>1514</v>
       </c>
-      <c r="I39" s="2">
+      <c r="I39" s="28">
         <v>556</v>
       </c>
-      <c r="K39" s="2">
+      <c r="J39" s="28"/>
+      <c r="K39" s="28">
         <v>1035</v>
       </c>
       <c r="O39" s="10" t="s">
@@ -9307,7 +9437,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="40" spans="1:16">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>39</v>
       </c>
@@ -9326,13 +9456,14 @@
       <c r="G40" s="2">
         <v>2025085</v>
       </c>
-      <c r="H40" s="2">
+      <c r="H40" s="28">
         <v>2566</v>
       </c>
-      <c r="I40" s="2">
+      <c r="I40" s="28">
         <v>1512</v>
       </c>
-      <c r="K40" s="2">
+      <c r="J40" s="28"/>
+      <c r="K40" s="28">
         <v>2039</v>
       </c>
       <c r="O40" s="10" t="s">
@@ -9342,7 +9473,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="41" spans="1:16">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>40</v>
       </c>
@@ -9356,18 +9487,20 @@
         <v>370</v>
       </c>
       <c r="E41" s="2">
-        <v>578</v>
+        <f>578-4.5</f>
+        <v>573.5</v>
       </c>
       <c r="G41" s="2">
         <v>2025086</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="28">
         <v>3538</v>
       </c>
-      <c r="I41" s="2">
+      <c r="I41" s="28">
         <v>2263</v>
       </c>
-      <c r="K41" s="2">
+      <c r="J41" s="28"/>
+      <c r="K41" s="28">
         <v>2900.5</v>
       </c>
       <c r="O41" s="10" t="s">
@@ -9377,7 +9510,7 @@
         <v>821</v>
       </c>
     </row>
-    <row r="42" spans="1:16">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>41</v>
       </c>
@@ -9396,13 +9529,14 @@
       <c r="G42" s="2">
         <v>2025087</v>
       </c>
-      <c r="H42" s="2">
+      <c r="H42" s="28">
         <v>1780</v>
       </c>
-      <c r="I42" s="2">
+      <c r="I42" s="28">
         <v>1728</v>
       </c>
-      <c r="K42" s="2">
+      <c r="J42" s="28"/>
+      <c r="K42" s="28">
         <v>1754</v>
       </c>
       <c r="O42" s="10" t="s">
@@ -9412,7 +9546,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="43" spans="1:16">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <v>42</v>
       </c>
@@ -9431,13 +9565,14 @@
       <c r="G43" s="2">
         <v>2025088</v>
       </c>
-      <c r="H43" s="2">
+      <c r="H43" s="28">
         <v>3113</v>
       </c>
-      <c r="I43" s="2">
+      <c r="I43" s="28">
         <v>899</v>
       </c>
-      <c r="K43" s="2">
+      <c r="J43" s="28"/>
+      <c r="K43" s="28">
         <v>2006</v>
       </c>
       <c r="O43" s="10" t="s">
@@ -9447,7 +9582,7 @@
         <v>951</v>
       </c>
     </row>
-    <row r="44" spans="1:16">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>43</v>
       </c>
@@ -9466,23 +9601,25 @@
       <c r="G44" s="2">
         <v>2025089</v>
       </c>
-      <c r="H44" s="2">
+      <c r="H44" s="28">
         <v>857</v>
       </c>
-      <c r="I44" s="2">
+      <c r="I44" s="28">
         <v>705</v>
       </c>
-      <c r="K44" s="2">
+      <c r="J44" s="28"/>
+      <c r="K44" s="28">
         <v>781</v>
       </c>
       <c r="O44" s="10" t="s">
         <v>263</v>
       </c>
       <c r="P44" s="10">
-        <v>578</v>
-      </c>
-    </row>
-    <row r="45" spans="1:16">
+        <f>578-4.5</f>
+        <v>573.5</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>44</v>
       </c>
@@ -9501,13 +9638,14 @@
       <c r="G45" s="2">
         <v>2025091</v>
       </c>
-      <c r="H45" s="2">
+      <c r="H45" s="28">
         <v>1230</v>
       </c>
-      <c r="I45" s="2">
+      <c r="I45" s="28">
         <v>990</v>
       </c>
-      <c r="K45" s="2">
+      <c r="J45" s="28"/>
+      <c r="K45" s="28">
         <v>1110</v>
       </c>
       <c r="O45" s="10" t="s">
@@ -9517,7 +9655,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="46" spans="1:16">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>45</v>
       </c>
@@ -9536,13 +9674,14 @@
       <c r="G46" s="2">
         <v>2025092</v>
       </c>
-      <c r="H46" s="2">
+      <c r="H46" s="28">
         <v>992</v>
       </c>
-      <c r="I46" s="2">
+      <c r="I46" s="28">
         <v>377</v>
       </c>
-      <c r="K46" s="2">
+      <c r="J46" s="28"/>
+      <c r="K46" s="28">
         <v>684.5</v>
       </c>
       <c r="O46" s="10" t="s">
@@ -9552,7 +9691,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="47" spans="1:16">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>46</v>
       </c>
@@ -9571,13 +9710,14 @@
       <c r="G47" s="2">
         <v>2025093</v>
       </c>
-      <c r="H47" s="2">
+      <c r="H47" s="28">
         <v>1076</v>
       </c>
-      <c r="I47" s="2">
+      <c r="I47" s="28">
         <v>803</v>
       </c>
-      <c r="K47" s="2">
+      <c r="J47" s="28"/>
+      <c r="K47" s="28">
         <v>939.5</v>
       </c>
       <c r="O47" s="10" t="s">
@@ -9587,7 +9727,7 @@
         <v>1476</v>
       </c>
     </row>
-    <row r="48" spans="1:16">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>47</v>
       </c>
@@ -9606,13 +9746,14 @@
       <c r="G48" s="2">
         <v>2025113</v>
       </c>
-      <c r="H48" s="2">
+      <c r="H48" s="28">
         <v>1876</v>
       </c>
-      <c r="I48" s="2">
+      <c r="I48" s="28">
         <v>608</v>
       </c>
-      <c r="K48" s="2">
+      <c r="J48" s="28"/>
+      <c r="K48" s="28">
         <v>1242</v>
       </c>
       <c r="O48" s="10" t="s">
@@ -9622,7 +9763,7 @@
         <v>1194</v>
       </c>
     </row>
-    <row r="49" spans="1:16">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>48</v>
       </c>
@@ -9641,14 +9782,15 @@
       <c r="G49" s="2">
         <v>2025115</v>
       </c>
-      <c r="H49" s="2">
-        <v>3982</v>
-      </c>
-      <c r="I49" s="2">
+      <c r="H49" s="28">
+        <v>3975.8</v>
+      </c>
+      <c r="I49" s="28">
         <v>2080</v>
       </c>
-      <c r="K49" s="2">
-        <v>3031</v>
+      <c r="J49" s="28"/>
+      <c r="K49" s="28">
+        <v>3027.9</v>
       </c>
       <c r="O49" s="10" t="s">
         <v>268</v>
@@ -9657,7 +9799,7 @@
         <v>1220</v>
       </c>
     </row>
-    <row r="50" spans="1:16">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
         <v>49</v>
       </c>
@@ -9676,13 +9818,14 @@
       <c r="G50" s="2">
         <v>2025116</v>
       </c>
-      <c r="H50" s="2">
+      <c r="H50" s="28">
         <v>3531</v>
       </c>
-      <c r="I50" s="2">
+      <c r="I50" s="28">
         <v>2364</v>
       </c>
-      <c r="K50" s="2">
+      <c r="J50" s="28"/>
+      <c r="K50" s="28">
         <v>2947.5</v>
       </c>
       <c r="O50" s="10" t="s">
@@ -9692,7 +9835,7 @@
         <v>2529</v>
       </c>
     </row>
-    <row r="51" spans="1:16">
+    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>50</v>
       </c>
@@ -9711,13 +9854,14 @@
       <c r="G51" s="2">
         <v>2025117</v>
       </c>
-      <c r="H51" s="2">
+      <c r="H51" s="28">
         <v>750</v>
       </c>
-      <c r="I51" s="2">
+      <c r="I51" s="28">
         <v>345</v>
       </c>
-      <c r="K51" s="2">
+      <c r="J51" s="28"/>
+      <c r="K51" s="28">
         <v>547.5</v>
       </c>
       <c r="O51" s="26" t="s">
@@ -9727,7 +9871,7 @@
         <v>1701</v>
       </c>
     </row>
-    <row r="52" spans="1:16">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>51</v>
       </c>
@@ -9746,13 +9890,14 @@
       <c r="G52" s="2">
         <v>2025119</v>
       </c>
-      <c r="H52" s="2">
+      <c r="H52" s="28">
         <v>754</v>
       </c>
-      <c r="I52" s="2">
+      <c r="I52" s="28">
         <v>582</v>
       </c>
-      <c r="K52" s="2">
+      <c r="J52" s="28"/>
+      <c r="K52" s="28">
         <v>668</v>
       </c>
       <c r="O52" s="26" t="s">
@@ -9762,7 +9907,7 @@
         <v>1821</v>
       </c>
     </row>
-    <row r="53" spans="1:16">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
         <v>52</v>
       </c>
@@ -9781,13 +9926,14 @@
       <c r="G53" s="2">
         <v>2025120</v>
       </c>
-      <c r="H53" s="2">
+      <c r="H53" s="28">
         <v>12</v>
       </c>
-      <c r="I53" s="2">
+      <c r="I53" s="28">
         <v>118</v>
       </c>
-      <c r="K53" s="2">
+      <c r="J53" s="28"/>
+      <c r="K53" s="28">
         <v>65</v>
       </c>
       <c r="O53" s="10" t="s">
@@ -9797,7 +9943,7 @@
         <v>1415</v>
       </c>
     </row>
-    <row r="54" spans="1:16">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
         <v>53</v>
       </c>
@@ -9816,13 +9962,14 @@
       <c r="G54" s="2">
         <v>2025121</v>
       </c>
-      <c r="H54" s="2">
-        <v>0</v>
-      </c>
-      <c r="I54" s="2">
-        <v>0</v>
-      </c>
-      <c r="K54" s="2">
+      <c r="H54" s="28">
+        <v>0</v>
+      </c>
+      <c r="I54" s="28">
+        <v>0</v>
+      </c>
+      <c r="J54" s="28"/>
+      <c r="K54" s="28">
         <v>0</v>
       </c>
       <c r="O54" s="10" t="s">
@@ -9832,7 +9979,7 @@
         <v>833</v>
       </c>
     </row>
-    <row r="55" spans="1:16">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
         <v>54</v>
       </c>
@@ -9851,13 +9998,14 @@
       <c r="G55" s="2">
         <v>2025122</v>
       </c>
-      <c r="H55" s="2">
+      <c r="H55" s="28">
         <v>2650</v>
       </c>
-      <c r="I55" s="2">
+      <c r="I55" s="28">
         <v>1147</v>
       </c>
-      <c r="K55" s="2">
+      <c r="J55" s="28"/>
+      <c r="K55" s="28">
         <v>1898.5</v>
       </c>
       <c r="O55" s="10" t="s">
@@ -9867,7 +10015,7 @@
         <v>1552</v>
       </c>
     </row>
-    <row r="56" spans="1:16">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
         <v>55</v>
       </c>
@@ -9886,13 +10034,14 @@
       <c r="G56" s="2">
         <v>2025123</v>
       </c>
-      <c r="H56" s="2">
-        <v>0</v>
-      </c>
-      <c r="I56" s="2">
-        <v>0</v>
-      </c>
-      <c r="K56" s="2">
+      <c r="H56" s="28">
+        <v>0</v>
+      </c>
+      <c r="I56" s="28">
+        <v>0</v>
+      </c>
+      <c r="J56" s="28"/>
+      <c r="K56" s="28">
         <v>0</v>
       </c>
       <c r="O56" s="10" t="s">
@@ -9902,7 +10051,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="57" spans="1:16">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
         <v>56</v>
       </c>
@@ -9921,13 +10070,14 @@
       <c r="G57" s="2">
         <v>2025124</v>
       </c>
-      <c r="H57" s="2">
+      <c r="H57" s="28">
         <v>2564</v>
       </c>
-      <c r="I57" s="2">
+      <c r="I57" s="28">
         <v>2102</v>
       </c>
-      <c r="K57" s="2">
+      <c r="J57" s="28"/>
+      <c r="K57" s="28">
         <v>2333</v>
       </c>
       <c r="O57" s="10" t="s">
@@ -9937,7 +10087,7 @@
         <v>2799</v>
       </c>
     </row>
-    <row r="58" spans="1:16">
+    <row r="58" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
         <v>57</v>
       </c>
@@ -9956,13 +10106,14 @@
       <c r="G58" s="2">
         <v>2025125</v>
       </c>
-      <c r="H58" s="2">
+      <c r="H58" s="28">
         <v>1891</v>
       </c>
-      <c r="I58" s="2">
+      <c r="I58" s="28">
         <v>891</v>
       </c>
-      <c r="K58" s="2">
+      <c r="J58" s="28"/>
+      <c r="K58" s="28">
         <v>1391</v>
       </c>
       <c r="O58" s="10" t="s">
@@ -9972,7 +10123,7 @@
         <v>1299</v>
       </c>
     </row>
-    <row r="59" spans="1:16">
+    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
         <v>58</v>
       </c>
@@ -9991,13 +10142,14 @@
       <c r="G59" s="2">
         <v>2025126</v>
       </c>
-      <c r="H59" s="2">
+      <c r="H59" s="28">
         <v>2057</v>
       </c>
-      <c r="I59" s="2">
+      <c r="I59" s="28">
         <v>1686</v>
       </c>
-      <c r="K59" s="2">
+      <c r="J59" s="28"/>
+      <c r="K59" s="28">
         <v>1871.5</v>
       </c>
       <c r="O59" s="10" t="s">
@@ -10007,7 +10159,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="60" spans="1:16">
+    <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>59</v>
       </c>
@@ -10026,13 +10178,14 @@
       <c r="G60" s="2">
         <v>2025127</v>
       </c>
-      <c r="H60" s="2">
+      <c r="H60" s="28">
         <v>926</v>
       </c>
-      <c r="I60" s="2">
+      <c r="I60" s="28">
         <v>1187</v>
       </c>
-      <c r="K60" s="2">
+      <c r="J60" s="28"/>
+      <c r="K60" s="28">
         <v>1056.5</v>
       </c>
       <c r="O60" s="10" t="s">
@@ -10042,7 +10195,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="61" spans="1:16">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
         <v>60</v>
       </c>
@@ -10061,13 +10214,14 @@
       <c r="G61" s="2">
         <v>2025128</v>
       </c>
-      <c r="H61" s="2">
+      <c r="H61" s="28">
         <v>2434</v>
       </c>
-      <c r="I61" s="2">
+      <c r="I61" s="28">
         <v>1076</v>
       </c>
-      <c r="K61" s="2">
+      <c r="J61" s="28"/>
+      <c r="K61" s="28">
         <v>1755</v>
       </c>
       <c r="O61" s="10" t="s">
@@ -10077,7 +10231,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="62" spans="1:16">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
         <v>61</v>
       </c>
@@ -10096,13 +10250,14 @@
       <c r="G62" s="2">
         <v>2025130</v>
       </c>
-      <c r="H62" s="2">
-        <v>0</v>
-      </c>
-      <c r="I62" s="2">
+      <c r="H62" s="28">
+        <v>0</v>
+      </c>
+      <c r="I62" s="28">
         <v>125</v>
       </c>
-      <c r="K62" s="2">
+      <c r="J62" s="28"/>
+      <c r="K62" s="28">
         <v>62.5</v>
       </c>
       <c r="O62" s="10" t="s">
@@ -10112,7 +10267,7 @@
         <v>1025</v>
       </c>
     </row>
-    <row r="63" spans="1:16">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
         <v>62</v>
       </c>
@@ -10131,13 +10286,14 @@
       <c r="G63" s="2">
         <v>2025132</v>
       </c>
-      <c r="H63" s="2">
+      <c r="H63" s="28">
         <v>821</v>
       </c>
-      <c r="I63" s="2">
+      <c r="I63" s="28">
         <v>561</v>
       </c>
-      <c r="K63" s="2">
+      <c r="J63" s="28"/>
+      <c r="K63" s="28">
         <v>691</v>
       </c>
       <c r="O63" s="20" t="s">
@@ -10147,7 +10303,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="64" spans="1:16">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>63</v>
       </c>
@@ -10166,14 +10322,15 @@
       <c r="G64" s="2">
         <v>2025133</v>
       </c>
-      <c r="H64" s="2">
+      <c r="H64" s="28">
         <v>951</v>
       </c>
-      <c r="I64" s="2">
-        <v>578</v>
-      </c>
-      <c r="K64" s="2">
-        <v>764.5</v>
+      <c r="I64" s="28">
+        <v>573.5</v>
+      </c>
+      <c r="J64" s="28"/>
+      <c r="K64" s="28">
+        <v>762.25</v>
       </c>
       <c r="O64" s="20" t="s">
         <v>283</v>
@@ -10182,7 +10339,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="65" spans="1:16">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
         <v>64</v>
       </c>
@@ -10201,13 +10358,14 @@
       <c r="G65" s="2">
         <v>2025134</v>
       </c>
-      <c r="H65" s="2">
+      <c r="H65" s="28">
         <v>12</v>
       </c>
-      <c r="I65" s="2">
-        <v>0</v>
-      </c>
-      <c r="K65" s="2">
+      <c r="I65" s="28">
+        <v>0</v>
+      </c>
+      <c r="J65" s="28"/>
+      <c r="K65" s="28">
         <v>6</v>
       </c>
       <c r="O65" s="10" t="s">
@@ -10217,7 +10375,7 @@
         <v>931</v>
       </c>
     </row>
-    <row r="66" spans="1:16">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
         <v>65</v>
       </c>
@@ -10236,13 +10394,14 @@
       <c r="G66" s="2">
         <v>2025137</v>
       </c>
-      <c r="H66" s="2">
+      <c r="H66" s="28">
         <v>1476</v>
       </c>
-      <c r="I66" s="2">
+      <c r="I66" s="28">
         <v>1194</v>
       </c>
-      <c r="K66" s="2">
+      <c r="J66" s="28"/>
+      <c r="K66" s="28">
         <v>1335</v>
       </c>
       <c r="O66" s="10" t="s">
@@ -10252,7 +10411,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="67" spans="1:16">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
         <v>66</v>
       </c>
@@ -10271,13 +10430,14 @@
       <c r="G67" s="2">
         <v>2025138</v>
       </c>
-      <c r="H67" s="2">
+      <c r="H67" s="28">
         <v>1220</v>
       </c>
-      <c r="I67" s="2">
+      <c r="I67" s="28">
         <v>2529</v>
       </c>
-      <c r="K67" s="2">
+      <c r="J67" s="28"/>
+      <c r="K67" s="28">
         <v>1874.5</v>
       </c>
       <c r="O67" s="10" t="s">
@@ -10287,7 +10447,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="68" spans="1:16">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A68" s="2">
         <v>67</v>
       </c>
@@ -10301,18 +10461,20 @@
         <v>369</v>
       </c>
       <c r="E68" s="2">
-        <v>977</v>
+        <f>977-106</f>
+        <v>871</v>
       </c>
       <c r="G68" s="2">
         <v>2025140</v>
       </c>
-      <c r="H68" s="2">
+      <c r="H68" s="28">
         <v>1415</v>
       </c>
-      <c r="I68" s="2">
+      <c r="I68" s="28">
         <v>833</v>
       </c>
-      <c r="K68" s="2">
+      <c r="J68" s="28"/>
+      <c r="K68" s="28">
         <v>1124</v>
       </c>
       <c r="O68" s="10" t="s">
@@ -10322,7 +10484,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="69" spans="1:16">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
         <v>68</v>
       </c>
@@ -10341,13 +10503,14 @@
       <c r="G69" s="2">
         <v>2025141</v>
       </c>
-      <c r="H69" s="2">
+      <c r="H69" s="28">
         <v>1552</v>
       </c>
-      <c r="I69" s="2">
+      <c r="I69" s="28">
         <v>561</v>
       </c>
-      <c r="K69" s="2">
+      <c r="J69" s="28"/>
+      <c r="K69" s="28">
         <v>1056.5</v>
       </c>
       <c r="O69" s="26" t="s">
@@ -10357,7 +10520,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="70" spans="1:16">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A70" s="2">
         <v>69</v>
       </c>
@@ -10376,13 +10539,14 @@
       <c r="G70" s="2">
         <v>2025142</v>
       </c>
-      <c r="H70" s="2">
+      <c r="H70" s="28">
         <v>2799</v>
       </c>
-      <c r="I70" s="2">
+      <c r="I70" s="28">
         <v>1299</v>
       </c>
-      <c r="K70" s="2">
+      <c r="J70" s="28"/>
+      <c r="K70" s="28">
         <v>2049</v>
       </c>
       <c r="O70" s="26" t="s">
@@ -10392,7 +10556,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="71" spans="1:16">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A71" s="2">
         <v>70</v>
       </c>
@@ -10411,23 +10575,25 @@
       <c r="G71" s="2">
         <v>2025148</v>
       </c>
-      <c r="H71" s="2">
+      <c r="H71" s="28">
         <v>392</v>
       </c>
-      <c r="I71" s="2">
+      <c r="I71" s="28">
         <v>156</v>
       </c>
-      <c r="K71" s="2">
+      <c r="J71" s="28"/>
+      <c r="K71" s="28">
         <v>274</v>
       </c>
       <c r="O71" s="25" t="s">
         <v>290</v>
       </c>
       <c r="P71" s="25">
-        <v>977</v>
-      </c>
-    </row>
-    <row r="72" spans="1:16">
+        <f>977-106</f>
+        <v>871</v>
+      </c>
+    </row>
+    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
         <v>71</v>
       </c>
@@ -10446,13 +10612,14 @@
       <c r="G72" s="2">
         <v>2025149</v>
       </c>
-      <c r="H72" s="2">
+      <c r="H72" s="28">
         <v>465</v>
       </c>
-      <c r="I72" s="2">
+      <c r="I72" s="28">
         <v>1025</v>
       </c>
-      <c r="K72" s="2">
+      <c r="J72" s="28"/>
+      <c r="K72" s="28">
         <v>745</v>
       </c>
       <c r="O72" s="25" t="s">
@@ -10462,7 +10629,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="73" spans="1:16">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A73" s="2">
         <v>72</v>
       </c>
@@ -10481,13 +10648,14 @@
       <c r="G73" s="2">
         <v>2025150</v>
       </c>
-      <c r="H73" s="2">
+      <c r="H73" s="28">
         <v>931</v>
       </c>
-      <c r="I73" s="2">
+      <c r="I73" s="28">
         <v>712</v>
       </c>
-      <c r="K73" s="2">
+      <c r="J73" s="28"/>
+      <c r="K73" s="28">
         <v>821.5</v>
       </c>
       <c r="O73" s="25" t="s">
@@ -10497,7 +10665,7 @@
         <v>994</v>
       </c>
     </row>
-    <row r="74" spans="1:16">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A74" s="2">
         <v>73</v>
       </c>
@@ -10516,13 +10684,14 @@
       <c r="G74" s="2">
         <v>2025151</v>
       </c>
-      <c r="H74" s="2">
+      <c r="H74" s="28">
         <v>510</v>
       </c>
-      <c r="I74" s="2">
+      <c r="I74" s="28">
         <v>557</v>
       </c>
-      <c r="K74" s="2">
+      <c r="J74" s="28"/>
+      <c r="K74" s="28">
         <v>533.5</v>
       </c>
       <c r="O74" s="25" t="s">
@@ -10532,7 +10701,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="75" spans="1:16">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A75" s="2">
         <v>74</v>
       </c>
@@ -10551,6 +10720,10 @@
       <c r="G75" s="2" t="s">
         <v>382</v>
       </c>
+      <c r="H75" s="28"/>
+      <c r="I75" s="28"/>
+      <c r="J75" s="28"/>
+      <c r="K75" s="28"/>
       <c r="O75" s="26" t="s">
         <v>294</v>
       </c>
@@ -10558,7 +10731,7 @@
         <v>2523</v>
       </c>
     </row>
-    <row r="76" spans="1:16">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A76" s="2">
         <v>75</v>
       </c>
@@ -10577,13 +10750,14 @@
       <c r="G76" s="2">
         <v>2025032</v>
       </c>
-      <c r="H76" s="2">
-        <v>0</v>
-      </c>
-      <c r="I76" s="2">
-        <v>0</v>
-      </c>
-      <c r="K76" s="2">
+      <c r="H76" s="28">
+        <v>0</v>
+      </c>
+      <c r="I76" s="28">
+        <v>0</v>
+      </c>
+      <c r="J76" s="28"/>
+      <c r="K76" s="28">
         <v>0</v>
       </c>
       <c r="O76" s="26" t="s">
@@ -10593,7 +10767,7 @@
         <v>1219</v>
       </c>
     </row>
-    <row r="77" spans="1:16">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A77" s="2">
         <v>76</v>
       </c>
@@ -10612,13 +10786,14 @@
       <c r="G77" s="2">
         <v>2025033</v>
       </c>
-      <c r="H77" s="2">
-        <v>0</v>
-      </c>
-      <c r="I77" s="2">
-        <v>0</v>
-      </c>
-      <c r="K77" s="2">
+      <c r="H77" s="28">
+        <v>0</v>
+      </c>
+      <c r="I77" s="28">
+        <v>0</v>
+      </c>
+      <c r="J77" s="28"/>
+      <c r="K77" s="28">
         <v>0</v>
       </c>
       <c r="O77" s="22" t="s">
@@ -10628,7 +10803,7 @@
         <v>2695</v>
       </c>
     </row>
-    <row r="78" spans="1:16">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A78" s="2">
         <v>77</v>
       </c>
@@ -10647,13 +10822,14 @@
       <c r="G78" s="2">
         <v>2025001</v>
       </c>
-      <c r="H78" s="2">
-        <v>0</v>
-      </c>
-      <c r="I78" s="2">
-        <v>0</v>
-      </c>
-      <c r="K78" s="2">
+      <c r="H78" s="28">
+        <v>0</v>
+      </c>
+      <c r="I78" s="28">
+        <v>0</v>
+      </c>
+      <c r="J78" s="28"/>
+      <c r="K78" s="28">
         <v>0</v>
       </c>
       <c r="O78" s="22" t="s">
@@ -10663,7 +10839,7 @@
         <v>1160</v>
       </c>
     </row>
-    <row r="79" spans="1:16">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A79" s="2">
         <v>78</v>
       </c>
@@ -10682,13 +10858,14 @@
       <c r="G79" s="2">
         <v>2025002</v>
       </c>
-      <c r="H79" s="2">
-        <v>0</v>
-      </c>
-      <c r="I79" s="2">
-        <v>0</v>
-      </c>
-      <c r="K79" s="2">
+      <c r="H79" s="28">
+        <v>0</v>
+      </c>
+      <c r="I79" s="28">
+        <v>0</v>
+      </c>
+      <c r="J79" s="28"/>
+      <c r="K79" s="28">
         <v>0</v>
       </c>
       <c r="O79" s="24" t="s">
@@ -10698,7 +10875,7 @@
         <v>933</v>
       </c>
     </row>
-    <row r="80" spans="1:16">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A80" s="2">
         <v>79</v>
       </c>
@@ -10717,13 +10894,14 @@
       <c r="G80" s="2">
         <v>2025020</v>
       </c>
-      <c r="H80" s="2">
-        <v>0</v>
-      </c>
-      <c r="I80" s="2">
-        <v>0</v>
-      </c>
-      <c r="K80" s="2">
+      <c r="H80" s="28">
+        <v>0</v>
+      </c>
+      <c r="I80" s="28">
+        <v>0</v>
+      </c>
+      <c r="J80" s="28"/>
+      <c r="K80" s="28">
         <v>0</v>
       </c>
       <c r="O80" s="24" t="s">
@@ -10733,7 +10911,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="81" spans="1:16">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A81" s="2">
         <v>80</v>
       </c>
@@ -10752,13 +10930,14 @@
       <c r="G81" s="2">
         <v>2025039</v>
       </c>
-      <c r="H81" s="2">
-        <v>0</v>
-      </c>
-      <c r="I81" s="2">
-        <v>0</v>
-      </c>
-      <c r="K81" s="2">
+      <c r="H81" s="28">
+        <v>0</v>
+      </c>
+      <c r="I81" s="28">
+        <v>0</v>
+      </c>
+      <c r="J81" s="28"/>
+      <c r="K81" s="28">
         <v>0</v>
       </c>
       <c r="O81" s="22" t="s">
@@ -10768,7 +10947,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="82" spans="1:16">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A82" s="2">
         <v>81</v>
       </c>
@@ -10787,13 +10966,14 @@
       <c r="G82" s="2">
         <v>2025114</v>
       </c>
-      <c r="H82" s="2">
-        <v>0</v>
-      </c>
-      <c r="I82" s="2">
-        <v>0</v>
-      </c>
-      <c r="K82" s="2">
+      <c r="H82" s="28">
+        <v>0</v>
+      </c>
+      <c r="I82" s="28">
+        <v>0</v>
+      </c>
+      <c r="J82" s="28"/>
+      <c r="K82" s="28">
         <v>0</v>
       </c>
       <c r="O82" s="22" t="s">
@@ -10803,7 +10983,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="83" spans="1:16">
+    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A83" s="2">
         <v>82</v>
       </c>
@@ -10822,13 +11002,14 @@
       <c r="G83" s="2">
         <v>2025135</v>
       </c>
-      <c r="H83" s="2">
-        <v>0</v>
-      </c>
-      <c r="I83" s="2">
-        <v>0</v>
-      </c>
-      <c r="K83" s="2">
+      <c r="H83" s="28">
+        <v>0</v>
+      </c>
+      <c r="I83" s="28">
+        <v>0</v>
+      </c>
+      <c r="J83" s="28"/>
+      <c r="K83" s="28">
         <v>0</v>
       </c>
       <c r="O83" s="26" t="s">
@@ -10838,7 +11019,7 @@
         <v>2790</v>
       </c>
     </row>
-    <row r="84" spans="1:16">
+    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A84" s="2">
         <v>83</v>
       </c>
@@ -10852,18 +11033,20 @@
         <v>369</v>
       </c>
       <c r="E84" s="2">
-        <v>2237</v>
+        <f>2237-66</f>
+        <v>2171</v>
       </c>
       <c r="G84" s="2">
         <v>2025131</v>
       </c>
-      <c r="H84" s="2">
+      <c r="H84" s="28">
         <v>1040</v>
       </c>
-      <c r="I84" s="2">
+      <c r="I84" s="28">
         <v>1642</v>
       </c>
-      <c r="K84" s="2">
+      <c r="J84" s="28"/>
+      <c r="K84" s="28">
         <v>1341</v>
       </c>
       <c r="O84" s="26" t="s">
@@ -10873,7 +11056,7 @@
         <v>888</v>
       </c>
     </row>
-    <row r="85" spans="1:16">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A85" s="2">
         <v>84</v>
       </c>
@@ -10887,18 +11070,20 @@
         <v>370</v>
       </c>
       <c r="E85" s="2">
-        <v>951</v>
+        <f>951-18</f>
+        <v>933</v>
       </c>
       <c r="G85" s="2">
         <v>2025136</v>
       </c>
-      <c r="H85" s="2">
+      <c r="H85" s="28">
         <v>1396</v>
       </c>
-      <c r="I85" s="2">
+      <c r="I85" s="28">
         <v>916</v>
       </c>
-      <c r="K85" s="2">
+      <c r="J85" s="28"/>
+      <c r="K85" s="28">
         <v>1156</v>
       </c>
       <c r="O85" s="26" t="s">
@@ -10908,7 +11093,7 @@
         <v>2113</v>
       </c>
     </row>
-    <row r="86" spans="1:16">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A86" s="2">
         <v>85</v>
       </c>
@@ -10927,13 +11112,14 @@
       <c r="G86" s="2">
         <v>2025111</v>
       </c>
-      <c r="H86" s="2">
+      <c r="H86" s="28">
         <v>1483</v>
       </c>
-      <c r="I86" s="2">
+      <c r="I86" s="28">
         <v>770</v>
       </c>
-      <c r="K86" s="2">
+      <c r="J86" s="28"/>
+      <c r="K86" s="28">
         <v>1126.5</v>
       </c>
       <c r="O86" s="26" t="s">
@@ -10943,7 +11129,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="87" spans="1:16">
+    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A87" s="2">
         <v>86</v>
       </c>
@@ -10962,23 +11148,25 @@
       <c r="G87" s="2">
         <v>2025139</v>
       </c>
-      <c r="H87" s="2">
+      <c r="H87" s="28">
         <v>780</v>
       </c>
-      <c r="I87" s="2">
+      <c r="I87" s="28">
         <v>557</v>
       </c>
-      <c r="K87" s="2">
+      <c r="J87" s="28"/>
+      <c r="K87" s="28">
         <v>668.5</v>
       </c>
       <c r="O87" s="22" t="s">
         <v>306</v>
       </c>
       <c r="P87" s="22">
-        <v>2237</v>
-      </c>
-    </row>
-    <row r="88" spans="1:16">
+        <f>2237-66</f>
+        <v>2171</v>
+      </c>
+    </row>
+    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A88" s="2">
         <v>87</v>
       </c>
@@ -10997,23 +11185,25 @@
       <c r="G88" s="2">
         <v>2025129</v>
       </c>
-      <c r="H88" s="2">
+      <c r="H88" s="28">
         <v>1517</v>
       </c>
-      <c r="I88" s="2">
+      <c r="I88" s="28">
         <v>811</v>
       </c>
-      <c r="K88" s="2">
+      <c r="J88" s="28"/>
+      <c r="K88" s="28">
         <v>1164</v>
       </c>
       <c r="O88" s="22" t="s">
         <v>307</v>
       </c>
       <c r="P88" s="22">
-        <v>951</v>
-      </c>
-    </row>
-    <row r="89" spans="1:16">
+        <f>951-18</f>
+        <v>933</v>
+      </c>
+    </row>
+    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A89" s="2">
         <v>88</v>
       </c>
@@ -11032,13 +11222,14 @@
       <c r="G89" s="2">
         <v>2025112</v>
       </c>
-      <c r="H89" s="2">
+      <c r="H89" s="28">
         <v>718</v>
       </c>
-      <c r="I89" s="2">
+      <c r="I89" s="28">
         <v>512</v>
       </c>
-      <c r="K89" s="2">
+      <c r="J89" s="28"/>
+      <c r="K89" s="28">
         <v>615</v>
       </c>
       <c r="O89" s="20" t="s">
@@ -11048,7 +11239,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="90" spans="1:16">
+    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A90" s="2">
         <v>89</v>
       </c>
@@ -11067,13 +11258,14 @@
       <c r="G90" s="2">
         <v>2025090</v>
       </c>
-      <c r="H90" s="2">
+      <c r="H90" s="28">
         <v>1103</v>
       </c>
-      <c r="I90" s="2">
+      <c r="I90" s="28">
         <v>813</v>
       </c>
-      <c r="K90" s="2">
+      <c r="J90" s="28"/>
+      <c r="K90" s="28">
         <v>958</v>
       </c>
       <c r="O90" s="20" t="s">
@@ -11083,7 +11275,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="91" spans="1:16">
+    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A91" s="2">
         <v>90</v>
       </c>
@@ -11102,13 +11294,14 @@
       <c r="G91" s="2">
         <v>2025083</v>
       </c>
-      <c r="H91" s="2">
+      <c r="H91" s="28">
         <v>717</v>
       </c>
-      <c r="I91" s="2">
+      <c r="I91" s="28">
         <v>835</v>
       </c>
-      <c r="K91" s="2">
+      <c r="J91" s="28"/>
+      <c r="K91" s="28">
         <v>776</v>
       </c>
       <c r="O91" s="26" t="s">
@@ -11118,7 +11311,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="92" spans="1:16">
+    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A92" s="2">
         <v>91</v>
       </c>
@@ -11137,13 +11330,14 @@
       <c r="G92" s="2">
         <v>2025118</v>
       </c>
-      <c r="H92" s="2">
+      <c r="H92" s="28">
         <v>1378</v>
       </c>
-      <c r="I92" s="2">
+      <c r="I92" s="28">
         <v>929</v>
       </c>
-      <c r="K92" s="2">
+      <c r="J92" s="28"/>
+      <c r="K92" s="28">
         <v>1153.5</v>
       </c>
       <c r="O92" s="26" t="s">
@@ -11153,7 +11347,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="93" spans="1:16">
+    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A93" s="2">
         <v>92</v>
       </c>
@@ -11172,14 +11366,15 @@
       <c r="G93" s="2" t="s">
         <v>383</v>
       </c>
-      <c r="H93" s="2">
-        <v>1173.6179775280898</v>
-      </c>
-      <c r="I93" s="2">
-        <v>740.22471910112358</v>
-      </c>
-      <c r="K93" s="2">
-        <v>956.92134831460669</v>
+      <c r="H93" s="28">
+        <v>1171.5822471910112</v>
+      </c>
+      <c r="I93" s="28">
+        <v>739.57191011235943</v>
+      </c>
+      <c r="J93" s="28"/>
+      <c r="K93" s="28">
+        <v>955.57707865168538</v>
       </c>
       <c r="O93" s="25" t="s">
         <v>312</v>
@@ -11188,7 +11383,7 @@
         <v>2715</v>
       </c>
     </row>
-    <row r="94" spans="1:16">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A94" s="2">
         <v>93</v>
       </c>
@@ -11211,7 +11406,7 @@
         <v>1696</v>
       </c>
     </row>
-    <row r="95" spans="1:16">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A95" s="2">
         <v>94</v>
       </c>
@@ -11234,7 +11429,7 @@
         <v>1294</v>
       </c>
     </row>
-    <row r="96" spans="1:16">
+    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A96" s="2">
         <v>95</v>
       </c>
@@ -11257,7 +11452,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="97" spans="1:24">
+    <row r="97" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A97" s="2">
         <v>96</v>
       </c>
@@ -11280,7 +11475,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="98" spans="1:24">
+    <row r="98" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A98" s="2">
         <v>97</v>
       </c>
@@ -11303,7 +11498,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="99" spans="1:24">
+    <row r="99" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A99" s="2">
         <v>98</v>
       </c>
@@ -11326,7 +11521,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="100" spans="1:24">
+    <row r="100" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A100" s="2">
         <v>99</v>
       </c>
@@ -11340,7 +11535,8 @@
         <v>369</v>
       </c>
       <c r="E100" s="2">
-        <v>209</v>
+        <f>209-(2.14+0.84)</f>
+        <v>206.02</v>
       </c>
       <c r="O100" s="20" t="s">
         <v>319</v>
@@ -11349,7 +11545,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="101" spans="1:24">
+    <row r="101" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A101" s="2">
         <v>100</v>
       </c>
@@ -11363,7 +11559,8 @@
         <v>370</v>
       </c>
       <c r="E101" s="2">
-        <v>248</v>
+        <f>248-35.6</f>
+        <v>212.4</v>
       </c>
       <c r="O101" s="19" t="s">
         <v>320</v>
@@ -11372,7 +11569,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="102" spans="1:24">
+    <row r="102" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A102" s="2">
         <v>101</v>
       </c>
@@ -11395,7 +11592,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="103" spans="1:24">
+    <row r="103" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A103" s="2">
         <v>102</v>
       </c>
@@ -11415,10 +11612,11 @@
         <v>322</v>
       </c>
       <c r="P103" s="22">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="104" spans="1:24">
+        <f>209-(0.84+2.14)</f>
+        <v>206.02</v>
+      </c>
+    </row>
+    <row r="104" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A104" s="2">
         <v>103</v>
       </c>
@@ -11438,10 +11636,11 @@
         <v>323</v>
       </c>
       <c r="P104" s="22">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="105" spans="1:24">
+        <f>248-35.6</f>
+        <v>212.4</v>
+      </c>
+    </row>
+    <row r="105" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A105" s="2">
         <v>104</v>
       </c>
@@ -11464,7 +11663,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="106" spans="1:24">
+    <row r="106" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A106" s="2">
         <v>105</v>
       </c>
@@ -11489,7 +11688,7 @@
       <c r="W106" s="22"/>
       <c r="X106" s="22"/>
     </row>
-    <row r="107" spans="1:24">
+    <row r="107" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A107" s="2">
         <v>106</v>
       </c>
@@ -11514,7 +11713,7 @@
       <c r="W107" s="22"/>
       <c r="X107" s="22"/>
     </row>
-    <row r="108" spans="1:24">
+    <row r="108" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A108" s="2">
         <v>107</v>
       </c>
@@ -11539,7 +11738,7 @@
       <c r="U108" s="20"/>
       <c r="V108" s="20"/>
     </row>
-    <row r="109" spans="1:24">
+    <row r="109" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A109" s="2">
         <v>108</v>
       </c>
@@ -11564,7 +11763,7 @@
       <c r="U109" s="20"/>
       <c r="V109" s="20"/>
     </row>
-    <row r="110" spans="1:24">
+    <row r="110" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A110" s="2">
         <v>109</v>
       </c>
@@ -11587,7 +11786,7 @@
         <v>1381</v>
       </c>
     </row>
-    <row r="111" spans="1:24">
+    <row r="111" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A111" s="2">
         <v>110</v>
       </c>
@@ -11610,7 +11809,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="112" spans="1:24">
+    <row r="112" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A112" s="2">
         <v>111</v>
       </c>
@@ -11633,7 +11832,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="113" spans="1:16">
+    <row r="113" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A113" s="2">
         <v>112</v>
       </c>
@@ -11656,7 +11855,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="114" spans="1:16">
+    <row r="114" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A114" s="2">
         <v>113</v>
       </c>
@@ -11679,7 +11878,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="115" spans="1:16">
+    <row r="115" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A115" s="2">
         <v>114</v>
       </c>
@@ -11702,7 +11901,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="116" spans="1:16">
+    <row r="116" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A116" s="2">
         <v>115</v>
       </c>
@@ -11725,7 +11924,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="117" spans="1:16">
+    <row r="117" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A117" s="2">
         <v>116</v>
       </c>
@@ -11748,7 +11947,7 @@
         <v>2222</v>
       </c>
     </row>
-    <row r="118" spans="1:16">
+    <row r="118" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A118" s="2">
         <v>117</v>
       </c>
@@ -11771,7 +11970,7 @@
         <v>939</v>
       </c>
     </row>
-    <row r="119" spans="1:16">
+    <row r="119" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A119" s="2">
         <v>118</v>
       </c>
@@ -11794,7 +11993,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="120" spans="1:16">
+    <row r="120" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A120" s="2">
         <v>119</v>
       </c>
@@ -11817,7 +12016,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="121" spans="1:16">
+    <row r="121" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A121" s="2">
         <v>120</v>
       </c>
@@ -11840,7 +12039,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="122" spans="1:16">
+    <row r="122" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A122" s="2">
         <v>121</v>
       </c>
@@ -11863,7 +12062,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="123" spans="1:16">
+    <row r="123" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A123" s="2">
         <v>122</v>
       </c>
@@ -11886,7 +12085,7 @@
         <v>2745</v>
       </c>
     </row>
-    <row r="124" spans="1:16">
+    <row r="124" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A124" s="2">
         <v>123</v>
       </c>
@@ -11909,7 +12108,7 @@
         <v>1244</v>
       </c>
     </row>
-    <row r="125" spans="1:16">
+    <row r="125" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A125" s="2">
         <v>124</v>
       </c>
@@ -11932,7 +12131,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="126" spans="1:16">
+    <row r="126" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A126" s="2">
         <v>125</v>
       </c>
@@ -11955,7 +12154,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="127" spans="1:16">
+    <row r="127" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A127" s="2">
         <v>126</v>
       </c>
@@ -11978,7 +12177,7 @@
         <v>1514</v>
       </c>
     </row>
-    <row r="128" spans="1:16">
+    <row r="128" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A128" s="2">
         <v>127</v>
       </c>
@@ -12001,7 +12200,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="129" spans="1:16">
+    <row r="129" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A129" s="2">
         <v>128</v>
       </c>
@@ -12024,7 +12223,7 @@
         <v>2566</v>
       </c>
     </row>
-    <row r="130" spans="1:16">
+    <row r="130" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A130" s="2">
         <v>129</v>
       </c>
@@ -12047,7 +12246,7 @@
         <v>1512</v>
       </c>
     </row>
-    <row r="131" spans="1:16">
+    <row r="131" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A131" s="2">
         <v>130</v>
       </c>
@@ -12070,7 +12269,7 @@
         <v>3538</v>
       </c>
     </row>
-    <row r="132" spans="1:16">
+    <row r="132" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A132" s="2">
         <v>131</v>
       </c>
@@ -12093,7 +12292,7 @@
         <v>2263</v>
       </c>
     </row>
-    <row r="133" spans="1:16">
+    <row r="133" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A133" s="2">
         <v>132</v>
       </c>
@@ -12116,7 +12315,7 @@
         <v>1780</v>
       </c>
     </row>
-    <row r="134" spans="1:16">
+    <row r="134" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A134" s="2">
         <v>133</v>
       </c>
@@ -12139,7 +12338,7 @@
         <v>1728</v>
       </c>
     </row>
-    <row r="135" spans="1:16">
+    <row r="135" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A135" s="2">
         <v>134</v>
       </c>
@@ -12162,7 +12361,7 @@
         <v>3113</v>
       </c>
     </row>
-    <row r="136" spans="1:16">
+    <row r="136" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A136" s="2">
         <v>135</v>
       </c>
@@ -12185,7 +12384,7 @@
         <v>899</v>
       </c>
     </row>
-    <row r="137" spans="1:16">
+    <row r="137" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A137" s="2">
         <v>136</v>
       </c>
@@ -12208,7 +12407,7 @@
         <v>857</v>
       </c>
     </row>
-    <row r="138" spans="1:16">
+    <row r="138" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A138" s="2">
         <v>137</v>
       </c>
@@ -12231,7 +12430,7 @@
         <v>705</v>
       </c>
     </row>
-    <row r="139" spans="1:16">
+    <row r="139" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A139" s="2">
         <v>138</v>
       </c>
@@ -12254,7 +12453,7 @@
         <v>2418</v>
       </c>
     </row>
-    <row r="140" spans="1:16">
+    <row r="140" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A140" s="2">
         <v>139</v>
       </c>
@@ -12277,7 +12476,7 @@
         <v>1706</v>
       </c>
     </row>
-    <row r="141" spans="1:16">
+    <row r="141" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A141" s="2">
         <v>140</v>
       </c>
@@ -12300,7 +12499,7 @@
         <v>1230</v>
       </c>
     </row>
-    <row r="142" spans="1:16">
+    <row r="142" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A142" s="2">
         <v>141</v>
       </c>
@@ -12323,7 +12522,7 @@
         <v>990</v>
       </c>
     </row>
-    <row r="143" spans="1:16">
+    <row r="143" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A143" s="2">
         <v>142</v>
       </c>
@@ -12346,7 +12545,7 @@
         <v>992</v>
       </c>
     </row>
-    <row r="144" spans="1:16">
+    <row r="144" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A144" s="2">
         <v>143</v>
       </c>
@@ -12369,7 +12568,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="145" spans="1:16">
+    <row r="145" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A145" s="2">
         <v>144</v>
       </c>
@@ -12392,7 +12591,7 @@
         <v>1076</v>
       </c>
     </row>
-    <row r="146" spans="1:16">
+    <row r="146" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A146" s="2">
         <v>145</v>
       </c>
@@ -12412,7 +12611,7 @@
         <v>803</v>
       </c>
     </row>
-    <row r="147" spans="1:16">
+    <row r="147" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A147" s="2">
         <v>146</v>
       </c>
@@ -12432,7 +12631,7 @@
         <v>1377</v>
       </c>
     </row>
-    <row r="148" spans="1:16">
+    <row r="148" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A148" s="2">
         <v>147</v>
       </c>
@@ -12452,7 +12651,7 @@
         <v>1864</v>
       </c>
     </row>
-    <row r="149" spans="1:16">
+    <row r="149" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A149" s="2">
         <v>148</v>
       </c>
@@ -12466,7 +12665,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:16">
+    <row r="150" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A150" s="2">
         <v>149</v>
       </c>
@@ -12483,7 +12682,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="151" spans="1:16">
+    <row r="151" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A151" s="2">
         <v>150</v>
       </c>
@@ -12500,7 +12699,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="152" spans="1:16">
+    <row r="152" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A152" s="2">
         <v>151</v>
       </c>
@@ -12517,7 +12716,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="153" spans="1:16">
+    <row r="153" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A153" s="2">
         <v>152</v>
       </c>
@@ -12534,7 +12733,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="154" spans="1:16">
+    <row r="154" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A154" s="2">
         <v>153</v>
       </c>
@@ -12551,7 +12750,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="155" spans="1:16">
+    <row r="155" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A155" s="2">
         <v>154</v>
       </c>
@@ -12568,7 +12767,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="156" spans="1:16">
+    <row r="156" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A156" s="2">
         <v>155</v>
       </c>
@@ -12585,7 +12784,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="157" spans="1:16">
+    <row r="157" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A157" s="2">
         <v>156</v>
       </c>
@@ -12602,7 +12801,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="158" spans="1:16">
+    <row r="158" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A158" s="2">
         <v>157</v>
       </c>
@@ -12619,7 +12818,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="159" spans="1:16">
+    <row r="159" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A159" s="2">
         <v>158</v>
       </c>
@@ -12636,7 +12835,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="160" spans="1:16">
+    <row r="160" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A160" s="2">
         <v>159</v>
       </c>
@@ -12653,7 +12852,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="161" spans="1:6">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A161" s="2">
         <v>160</v>
       </c>
@@ -12670,7 +12869,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="162" spans="1:6">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A162" s="2">
         <v>161</v>
       </c>
@@ -12687,7 +12886,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="163" spans="1:6">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A163" s="2">
         <v>162</v>
       </c>
@@ -12704,7 +12903,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="164" spans="1:6">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A164" s="2">
         <v>163</v>
       </c>
@@ -12721,7 +12920,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="165" spans="1:6">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A165" s="2">
         <v>164</v>
       </c>
@@ -12738,7 +12937,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="166" spans="1:6">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A166" s="2">
         <v>165</v>
       </c>
@@ -12755,7 +12954,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="167" spans="1:6">
+    <row r="167" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A167" s="2">
         <v>166</v>
       </c>
@@ -12772,7 +12971,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="168" spans="1:6">
+    <row r="168" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A168" s="2">
         <v>167</v>
       </c>
@@ -12789,7 +12988,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="169" spans="1:6">
+    <row r="169" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A169" s="2">
         <v>168</v>
       </c>
@@ -12806,7 +13005,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="170" spans="1:6">
+    <row r="170" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A170" s="2">
         <v>169</v>
       </c>
@@ -12823,7 +13022,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="171" spans="1:6">
+    <row r="171" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A171" s="2">
         <v>170</v>
       </c>
@@ -12840,7 +13039,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="172" spans="1:6">
+    <row r="172" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A172" s="2">
         <v>171</v>
       </c>
@@ -12857,7 +13056,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="173" spans="1:6">
+    <row r="173" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A173" s="2">
         <v>172</v>
       </c>
@@ -12874,7 +13073,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="174" spans="1:6">
+    <row r="174" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A174" s="2">
         <v>173</v>
       </c>
@@ -12891,7 +13090,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="175" spans="1:6">
+    <row r="175" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A175" s="2">
         <v>174</v>
       </c>
@@ -12908,7 +13107,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="176" spans="1:6">
+    <row r="176" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A176" s="2">
         <v>175</v>
       </c>
@@ -12925,7 +13124,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="177" spans="1:6">
+    <row r="177" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A177" s="2">
         <v>176</v>
       </c>
@@ -12942,7 +13141,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="178" spans="1:6">
+    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A178" s="2">
         <v>177</v>
       </c>
@@ -12959,7 +13158,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="179" spans="1:6">
+    <row r="179" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C179" s="4">
         <v>2025118</v>
       </c>
@@ -12974,8 +13173,8 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F165" xr:uid="{60289AD6-9204-4C5F-9F5B-57B3483DE391}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F148">
+  <autoFilter ref="A1:F165"/>
+  <sortState ref="A2:F148">
     <sortCondition ref="A2:A148"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12983,9 +13182,9 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F933308-2D03-4466-9DB8-419CC3C4B7C8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>